<commit_message>
Daily construction lead update
</commit_message>
<xml_diff>
--- a/data/nyc_construction_leads.xlsx
+++ b/data/nyc_construction_leads.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,7 +493,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>40-38 189 STREET, Queens</t>
+          <t>211-07 34 ROAD, Queens</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -503,16 +503,16 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4038 EASTERN REALTY LLC</t>
+          <t>211-05 34TH RD REALTY LLC</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Pending CPE/ACPE Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -521,22 +521,22 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Q01466083-I1</t>
+          <t>Q01403320-S4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>PROPOSE A NEW TWO STORY WITH TWO FAMILY HOUSE. OBTAIN NEW C OF O.</t>
+          <t>FILE PL &amp; SP WORKTYPE IN CONJUNCTION WITH JOB#Q01403320</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>XIAOHONG</t>
+          <t>KAI</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>ZHAO</t>
+          <t>HUANG</t>
         </is>
       </c>
     </row>
@@ -551,17 +551,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>8-48 ASTORIA BOULEVARD, Queens</t>
+          <t>14 DOE PLACE, Staten Island</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Queens</t>
+          <t>Staten Island</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>MR. OLU COLE</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="G3" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -579,22 +579,22 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Q01450056-S4</t>
+          <t>S00965093-S6</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>MECHNICAL SYSTEM FOR NEW 7-STORY MONOLITHIC CONCRETE BUILDING</t>
+          <t>Installation of a 9' curb cut (6' cc with (2) 18" splays)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Roman</t>
+          <t>LALITH</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Sorokko</t>
+          <t>RAJAKARUNA</t>
         </is>
       </c>
     </row>
@@ -609,17 +609,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1663 EAST   18 STREET, Brooklyn</t>
+          <t>26-37 30 STREET, Queens</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Brooklyn</t>
+          <t>Queens</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>30th Street Property Holdings LLC</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="G4" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -637,22 +637,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>B01405960-S3</t>
+          <t>Q01385871-S2</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>INSTALL NEW MECHANICAL SYSTEM THROUGHOUT NEW 12-STORY MONOLITHIC CONCRETE BUILDING</t>
+          <t>INSTALLATION OF PLUMBING SYSTEM FOR ENTIRE BUILDING INCONJUNCTION WITH NB JOB #Q01385871-I1</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Roman</t>
+          <t>Dmitry</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Sorokko</t>
+          <t>Levin</t>
         </is>
       </c>
     </row>
@@ -667,17 +667,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>144 WILD AVENUE, Staten Island</t>
+          <t>8741 BAY   16 STREET, Brooklyn</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Staten Island</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -686,31 +686,31 @@
         </is>
       </c>
       <c r="G5" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>S01371873-I1</t>
+          <t>B01463420-I1</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>CONSTRUCT A TWO FAMILY RESIDENCE WITH ACCESSORY OFF-STREET PARKING FOR TWO CARS</t>
+          <t>PROPOSE A NEW THREE STORY WITH THREE FAMILY DWELLINGS FAMILY.  OBTAIN NEW C OF O.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Stanley</t>
+          <t>XIAOHONG</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Krebushevski</t>
+          <t>ZHAO</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>40-38 189 STREET, Queens</t>
+          <t>211-03 34 ROAD, Queens</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -735,16 +735,16 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>4038 EASTERN REALTY LLC</t>
+          <t>211-05 34TH RD REALTY LLC</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Pending Plan Examiner Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G6" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -753,217 +753,221 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Q01466083-S1</t>
+          <t>Q01403318-S4</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>FILE SOE IN CONJUNCTION WITH JOB#Q01466083</t>
+          <t>FILE PL &amp; SP WORKTYPE IN CONJUNCTION WITH JOB#Q01403318</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>XIAOHONG</t>
+          <t>KAI</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>ZHAO</t>
+          <t>HUANG</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alteration</t>
+          <t>New Building</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>783 QUINCY STREET, Brooklyn</t>
+          <t>211-05 34 ROAD, Queens</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Brooklyn</t>
+          <t>Queens</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>211-05 34TH RD REALTY LLC</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Pending CPE/ACPE Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G7" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>18000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>B01464808-I1</t>
+          <t>Q01404099-S4</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Repair of damaged brownstone and peeling plaster/paint on Exposure 1 facade</t>
+          <t>FILE PL &amp; SP WORKTYPE IN CONJUNCTION WITH JOB#Q01404099</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Sunil</t>
+          <t>KAI</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Saigal</t>
+          <t>HUANG</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alteration</t>
+          <t>New Building</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>200 WEST   57 STREET, Manhattan</t>
+          <t>2124 AVENUE P, Brooklyn</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Manhattan</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>The Feil Organization</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Pending CPE/ACPE Assignment</t>
+          <t>Pending Plan Examiner Assignment</t>
         </is>
       </c>
       <c r="G8" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>30000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>M01463256-S2</t>
+          <t>B01381870-S7</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>IOR ALTERATION WITHIN EXISTING TENANT SPACE STE 708 ON 7TH FLOOR IN EXISTING BUILDING: NEW PLUMBING FIXTURES PER NEW LAYOUT, NEW DENTAL PLUMBING FIXTURES PER DENTAL NEEDS, NEW ELECTRICAL HOT WATER HEATER, NO CHANGE TO OCCUPANCY, GROUP AND USE.</t>
+          <t>STRUCTURAL WORKS FOR NEW 12-STORY MONOLITHIC CONCRETE BUILDING</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>XIU</t>
+          <t>Roman</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>CHEN</t>
+          <t>Sorokko</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alteration</t>
+          <t>New Building</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>31-40 35 STREET, Queens</t>
+          <t>8743 BAY   16 STREET, Brooklyn</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Queens</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>Pending CPE/ACPE Assignment</t>
         </is>
       </c>
       <c r="G9" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>54550</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Q01462560-I1</t>
+          <t>B01463830-I1</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>INTERIOR RENOVATION OF EXISTING RESIDENTIAL APARTMENT TO UPDATE BEDROOM LAYOUT. NEW WALLS AND OUTLETS PER PLAN. NO CHANGE IN EGRESS, USE OR OCCUPANCY.</t>
+          <t>PROPOSE A NEW THREE STORY WITH THREE FAMILY DWELLING HOUSE. OBTAIN NEW C OF O.</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Kun</t>
+          <t>XIAOHONG</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Wu</t>
+          <t>ZHAO</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alteration</t>
+          <t>New Building</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>200 WEST   57 STREET, Manhattan</t>
+          <t>8745 BAY   16 STREET, Brooklyn</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Manhattan</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>The Feil Organization</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -972,31 +976,31 @@
         </is>
       </c>
       <c r="G10" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>15000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>M01463256-S1</t>
+          <t>B01463422-I1</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>INTERIOR ALTERATION WITHIN EXISTING TENANT SPACE STE 708 ON 7TH FLOOR IN EXISTING BUILDING: NEW VRF SYSTEM WITH ROOFTOP CONDENSER AND INDOOR AIR HANDLERS NEW FRESH AIR INTAKE SYSTEM NEW EXHAUST FAN SYSTEM NEW ASSOCIATED DUCTWORK, DIFFUSERS, AND PIPING.</t>
+          <t>PROPOSE A NEW THREE STORY WITH THREE FAMILY DWELLINGS HOUSE. OBTAIN NEW C OF O.</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>XIU</t>
+          <t>XIAOHONG</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>CHEN</t>
+          <t>ZHAO</t>
         </is>
       </c>
     </row>
@@ -1011,50 +1015,50 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>262 5 AVENUE, Manhattan</t>
+          <t>165 RUTLAND ROAD, Brooklyn</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Manhattan</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Doria Scaffolding LLC</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Pending Prof Cert QA Assignment</t>
+          <t>Pending CPE/ACPE Assignment</t>
         </is>
       </c>
       <c r="G11" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>15000</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>M01330105-S2</t>
+          <t>B01457959-I1</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>INSTALLATION OF TEMPORARY MATERIAL HOIST ON OUTRIGGERS PER PLAN SUBMITTED. WORK SHALL COMPLY WITH 2022 BUILDING CODE CHAPTER 33. NO CHANGE IN USE, EGRESS AND/OR OCCUPANCY WITH THIS APPLICATION.</t>
+          <t>APPLICATION FILE TO EXTERIOR FACADE REPAIR AS RECONSTRUCTION OF THE FRONT MASONRY, STAIR, SIDE CHEEK WALLS  AND CORNICE PAINTING AT FRONT ELEVATION. REMOVE VIOLATION# 39198431L.. NO CHANGE IN USE, EGRESS OR OCCUPANCY UNDER THIS APPLICATION.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>ZELJKO</t>
+          <t>Mumtaz</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>STEVANOVIC</t>
+          <t>Hussain</t>
         </is>
       </c>
     </row>
@@ -1069,50 +1073,50 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14 WEST  170 STREET, Bronx</t>
+          <t>341 KINGSBOROUGH    3 WALK, Brooklyn</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Bronx</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Latino Pastoral Action Center</t>
+          <t>NYCHA</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Pending CPE/ACPE Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>30000</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>X01464173-I1</t>
+          <t>B01455837-I1</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Removal of existing roof assembly down to existing structural metal roof deck and installation of new roof insulation and TPO roofing membrane system over existing structural metal roof deck. No change in use or occupancy. No structural work.</t>
+          <t>INSTALLATION OF TEMPORARY SIDEWALK SHED AT 341 KINGSBOROUGH 3 WALK, BROOKLYN, NY 11233 AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Marcus</t>
+          <t>WALIUR</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Royes</t>
+          <t>RAHMAN</t>
         </is>
       </c>
     </row>
@@ -1127,17 +1131,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>173 CANAL STREET, Manhattan</t>
+          <t>459 EAST  149 STREET, Bronx</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Manhattan</t>
+          <t>Bronx</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>RABER ENTERPRISES LLC</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1146,31 +1150,31 @@
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>100000</t>
+          <t>45000</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>M01462390-I1</t>
+          <t>X01038608-P1</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1ST FLOOR INTERIOR RENOVATION. REMOVE AND INSTALL NEW PARTITIONS. NO CHANGE IN USE, OCCUPANCY, OR EGRESS UNDER THIS APPLICATION.</t>
+          <t>RENOVATE EXISTING STORES, REMOVE NON BEARING PARTITIONS AND COUNTERS</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Ruoyu</t>
+          <t>Kenneth</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Wei</t>
+          <t>Koons</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1189,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>83-05 116 STREET, Queens</t>
+          <t>86-21 89 STREET, Queens</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1195,40 +1199,40 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>PARKSITE CONSTRUCTION CORP</t>
+          <t>GOLDEN ROCK 2026 LLC</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Pending Plan Examiner Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>45000</t>
+          <t>25000</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Q01462049-I1</t>
+          <t>Q01466154-I1</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>APPLICATION FILED FOR SUPPORT-OF-EXCAVATION FOR A NEW V15-6 CON EDISON VAULT UNDER THE SIDEWALK AT 83-05 116 STREET, QUEENS, NY</t>
+          <t>INTERIOR RENOVATION OF EXISTING CELLAR TO CURE ECB VIOLATIONS# 34232266L; 34458272J. NO CHANGE IN USE, OCCUPANCY OR EGRESS.</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>SAMER</t>
+          <t>LOUIS</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>ABOU-GHAIDA</t>
+          <t>KONG</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1247,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>45 SUTTON PLACE SOUTH, Manhattan</t>
+          <t>111 BROADWAY, Manhattan</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1251,38 +1255,42 @@
           <t>Manhattan</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>CAPITAL PROPERTIES</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Pending CPE/ACPE Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>20500</t>
+          <t>17280</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>M01463366-S1</t>
+          <t>M01386850-P1</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>renovate kitchen, replace bathroom fixtures and install new washing machine. no change in use, egress or occupancy.</t>
+          <t>SPRINKLER MODIFICATIONS TAKING PLACE ON 20TH FLOOR AS PER PLANS FILED HEREWITH. NO CHANGE IN USE, EGRESS, OR OCCUPANCY.</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Helge</t>
+          <t>Steven</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Fuhrmann</t>
+          <t>Snyder</t>
         </is>
       </c>
     </row>
@@ -1297,17 +1305,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>25 WASHINGTON SQUARE NORTH, Manhattan</t>
+          <t>127 KINGSBOROUGH    1 WALK, Brooklyn</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Manhattan</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>PYRAMID RESTORATION NY</t>
+          <t>NYCHA</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1316,31 +1324,31 @@
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>M01449368-I1</t>
+          <t>B01450003-I1</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>PROPOSED INSTALLATION OF TEMPORARY PIPE SCAFFOLD AS PER PLANS. WORK SHALL COMPLY WITH CHAPTER #33 OF 2022 THE NYC BUILDING CODE. NO CHANGE IN USE, OCCUPANCY, OR EGRESS UNDER THIS APPLICATION.</t>
+          <t>INSTALLATION OF NEW SIDEWALK SHED AT 127 KINGSBOROUGH 1 WALK BROOKLYN NY 11233 AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Charles</t>
+          <t>WALIUR</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Davidson</t>
+          <t>RAHMAN</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1363,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>663 ROGERS AVENUE, Brooklyn</t>
+          <t>171 EAST   93 STREET, Brooklyn</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1365,40 +1373,40 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>MICASAA</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Pending Prof Cert QA Assignment</t>
+          <t>Pending CPE/ACPE Assignment</t>
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>20000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>B01463979-I1</t>
+          <t>B01457449-S1</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>APPLICATION FILING TO INSTALL CONDENSING UNIT AT ROOF TOP AS PER PLAN. NO CHANGE OF USE, EGRESS AND OCCUPANCY UNDER THIS APPLICATION.</t>
+          <t>INTERIOR RENOVATION OF CELLAR. REMOVE KITCHEN AND BATHTUB INSTALL NEW BATHRROM. FIILE TO ADDRESS ECB VIOLATION 34275318Y</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>KAMRUL</t>
+          <t>Oswin</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>AHSAN</t>
+          <t>Fairweather</t>
         </is>
       </c>
     </row>
@@ -1413,7 +1421,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>63 PENNSYLVANIA AVENUE, Brooklyn</t>
+          <t>108 KINGSBORO    1 WALK, Brooklyn</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1423,7 +1431,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ROSE SHEPHERD MANAGEMENT</t>
+          <t>NYCHA</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1432,31 +1440,31 @@
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>12000</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>B00656210-P2</t>
+          <t>B01450001-I1</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Mechanical work as shown on plans</t>
+          <t>INSTALLATION OF NEW SIDEWALK SHED AT 108 KINGSBOROUGH 1 WALK BROOKLYN NY  11233 AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Evodia</t>
+          <t>WALIUR</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Ibrahim</t>
+          <t>RAHMAN</t>
         </is>
       </c>
     </row>
@@ -1471,12 +1479,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>107 WEST  132 STREET, Manhattan</t>
+          <t>171 EAST   93 STREET, Brooklyn</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Manhattan</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1486,35 +1494,35 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Pending Plan Examiner Assignment</t>
+          <t>Pending CPE/ACPE Assignment</t>
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>50000</t>
+          <t>45000</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>M01418005-S5</t>
+          <t>B01457449-I1</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>FRONT AND REAR FACADE RESTORATION WORK AS PER PLANS</t>
+          <t>INTERIOR RENOVATION OF CELLAR LEVEL. MINIOR PARTION WORK. REMOVE KITCHEN AND BATHTUB AND INSTALL NEW BATHROOM. FILE TO ADDRESS VIOLATION ECB 34275318Y.</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>JEFFREY</t>
+          <t>Oswin</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>BELL</t>
+          <t>Fairweather</t>
         </is>
       </c>
     </row>
@@ -1529,50 +1537,50 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>200 WEST   57 STREET, Manhattan</t>
+          <t>242 45 STREET, Brooklyn</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Manhattan</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>The Feil Organization</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Pending CPE/ACPE Assignment</t>
+          <t>Pending Plan Examiner Assignment</t>
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>121700</t>
+          <t>57500</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>M01463256-I1</t>
+          <t>B01459667-S1</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>INTERIOR ALTERATION WITHIN EXISTING TENANT SPACE STE 708 ON 7TH FLOOR IN EXISTING BUILDING: NEW NON-BEARING INTERIOR PARTITIONS, NEW INTERIOR FINISHES, NEW MILLWORK, NEW LIGHTING. NO CHANGE TO OCCUPANCY, GROUP AND USE.</t>
+          <t>NEW KITCHEN LAYOUT ON FIRST AND SECOND FLOORS, REPLACEMENT OF BATHROOM FIXTURES, EXISTING GAS METER 1 TO CONNECT TO EXISTING BOILER WITH INDIRECT TANK AND GAS RANGE ON FIRST FLOOR ONLY. EXISTING GAS METER 2 TO BE REMOVED</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>XIU</t>
+          <t>Laura</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>CHEN</t>
+          <t>Lievano</t>
         </is>
       </c>
     </row>
@@ -1587,17 +1595,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>40-38 189 STREET, Queens</t>
+          <t>308 KINGSBORO    3 WALK, Brooklyn</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Queens</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>4038 EASTERN REALTY LLC</t>
+          <t>NYCHA</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1606,31 +1614,31 @@
         </is>
       </c>
       <c r="G21" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Q01466129-I1</t>
+          <t>B01452530-I1</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>INSTALL 8' TEMPORARY CONSTRUCTION FENCE AT THE ABOVE ADDRESS</t>
+          <t>INSTALLATION OF NEW SIDEWALK SHED AT 308 KINGSBOROUGH 3 WALK BROOKLYN NY 11233  AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>KAI</t>
+          <t>WALIUR</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>HUANG</t>
+          <t>RAHMAN</t>
         </is>
       </c>
     </row>
@@ -1645,17 +1653,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>173 CANAL STREET, Manhattan</t>
+          <t>4137 3 AVENUE, Bronx</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Manhattan</t>
+          <t>Bronx</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>RABER ENTERPRISES LLC</t>
+          <t>RBA DEVELOPERS LLC</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1664,31 +1672,31 @@
         </is>
       </c>
       <c r="G22" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>21000</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>M01462390-S1</t>
+          <t>X01459199-I1</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>IST FLOOR INTERIOR RENOVATION. INSTALL PLUMBING FIXTURES. NO CHANGE IN USE, OCCUPANCY, OR EGRESS UNDER THIS APPLICATION.</t>
+          <t>Install plumbing systems in conjunction with NB X01223342-I1. There is no change in use, occupancy, or egress.</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Ruoyu</t>
+          <t>Gregory</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Wei</t>
+          <t>Mortman</t>
         </is>
       </c>
     </row>
@@ -1703,17 +1711,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>233 SOUTH    3 STREET, Brooklyn</t>
+          <t>1407 BROADWAY, Manhattan</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Brooklyn</t>
+          <t>Manhattan</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>GREENBROOK PARTNERS</t>
+          <t>SHORENSTEIN</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1722,31 +1730,31 @@
         </is>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>172500</t>
+          <t>180000</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>B01456715-I1</t>
+          <t>M01457423-I1</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Renovation to existing commercial first floor tenant space. New equipment and finishes for bakery build out. Add one door to existing storefront. Plumbing and HVAC filed subsequently</t>
+          <t>INTERIOR RENOVATIONS CONSISTING OF PARTITIONS AND FINISHES  AS PER PLANS FILED HEREWITH. NO  CHANGE TO USE, EGRESS OR OCCUPANCY</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Cortney</t>
+          <t>LEMUEL</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Walleston</t>
+          <t>GUIDOS</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1769,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>6645 BROADWAY, Bronx</t>
+          <t>1311 THIERIOT AVENUE, Bronx</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1771,40 +1779,40 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CEDARBRIDGE</t>
+          <t>CREPAS LLC</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Pending CPE/ACPE Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>60000</t>
+          <t>17000</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>X01462292-I1</t>
+          <t>X01462758-I1</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>PROPOSED TO REPAIR THE BOTTOM OF THE EXISTING STRUCTURAL FOR THE PART OF THE GARAGE AT CELLAR. REINFORCED CONCRETE SLAB,  SUPPORING THE FIRST FLOOR IN ADDITION TO CONCRETE ENCASEMENT FOR STRUCTURAL STEEL ELEMENTS. THERE IS NO CHANGE OCCUANCY, USE OR EGRES</t>
+          <t>Replace seven (7) steel window lintels facing the street and repoint facade cracks as necessary. No change in use, egress, or occupancy.</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Edwin</t>
+          <t>SAHAND</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Cheuk</t>
+          <t>AINECHI</t>
         </is>
       </c>
     </row>
@@ -1819,7 +1827,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>547 CLINTON STREET, Brooklyn</t>
+          <t>2303 AVENUE D, Brooklyn</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1838,31 +1846,31 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>75000</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>B01454896-P1</t>
+          <t>B01403876-P1</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>LEGALIZE THE REMOVAL OF ILLEGAL SPIRAL STAIRCASE BETWEEN 1ST AND 2ND FLOOR COMBING TWO APARTMENTS.  LEGALIZE THE INSTALLATION OF FIREBOX DAMPER AT 1ST FLOOR FIREPLACE.  THIS WILL ADDRESS DOB VIOLATION VW 110298C06MJ11.</t>
+          <t>Plumbing work in conjunction with interior renovation</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>REGINALD</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>THOMAS</t>
+          <t>MOSTAFA</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1885,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>45 SUTTON PLACE SOUTH, Manhattan</t>
+          <t>148 MADISON AVENUE, Manhattan</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1885,38 +1893,42 @@
           <t>Manhattan</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>GFP REAL ESTATE LLC</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Pending CPE/ACPE Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>147200</t>
+          <t>52500</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>M01463366-I1</t>
+          <t>M01399810-S2</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Renovation of Apartment 3J as per plans</t>
+          <t>Installation of new split heat pump and ventilation equipment for an existing commercial space.  No change of use, egress or occupancy under this application.</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Helge</t>
+          <t>Tyrone</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Fuhrmann</t>
+          <t>Wells</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1943,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>3520 TILDEN AVENUE, Brooklyn</t>
+          <t>342 KINGSBORO    3 WALK, Brooklyn</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1941,40 +1953,40 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>NYCHA</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Pending CPE/ACPE Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>B01459311-I1</t>
+          <t>B01452518-I1</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>FILING TO OBTAIN CERTIFICATE OF COMPLIANCE.  JOB PREVIOUSLY FILED UNDER JOB # B00552772-I1.  INITIAL SCOPE OF WORK WAS TO REPLACE THE CONDENSER ON THE ROOF.  NO ROPOSED WORK ON THIS APPLICATION.</t>
+          <t>INSTALLATION OF NEW SIDEWALK SHED AT 342 KINGSBOROUGH 3 WALK  BROOKLYN NY 11233 AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>KENNETH</t>
+          <t>WALIUR</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>PHILOGENE</t>
+          <t>RAHMAN</t>
         </is>
       </c>
     </row>
@@ -1989,50 +2001,50 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>118 NOEL ROAD, Queens</t>
+          <t>2675 PITKIN AVENUE, Brooklyn</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Queens</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Pending Prof Cert QA Assignment</t>
+          <t>Pending Plan Examiner Assignment</t>
         </is>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>25000</t>
+          <t>19000</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Q01465575-I1</t>
+          <t>B01330815-P1</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>LIFT OF EXISTING ONE FAMILY DWELLING UNIT</t>
+          <t>INTERIOR RENOVATION OF EXISTING COMMERCIAL SPACE FOR FOOD TAKEOUT INCLUDING CARPENTRY, NEW PARTITIONS, NEW COMMERCIAL KITCHEN, EXHAUST HOOD, FAN INSTALL. NO CHANGE IN USE, OCCUPANCY AND EGRESS IS INVOLVED UNDER THIS APPLICATION.</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>LEON</t>
+          <t>KARTIK</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SKVIRSKY</t>
+          <t>CHANDA</t>
         </is>
       </c>
     </row>
@@ -2047,7 +2059,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>306 SHERIDAN AVENUE, Brooklyn</t>
+          <t>584 KOSCIUSZKO STREET, Brooklyn</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2066,31 +2078,31 @@
         </is>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>20000</t>
+          <t>15000</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>B01463073-I1</t>
+          <t>B01433221-I1</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>AXMISAXJIWHD</t>
+          <t>Legalize installation of parking shed</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Mohammad</t>
+          <t>WILLIAM</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Alauddin</t>
+          <t>ROSS</t>
         </is>
       </c>
     </row>
@@ -2105,26 +2117,26 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>200 WEST   57 STREET, Manhattan</t>
+          <t>207 KINGSBORO    2 WALK, Brooklyn</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Manhattan</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>The Feil Organization</t>
+          <t>NYCHA</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Pending CPE/ACPE Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -2133,22 +2145,22 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>M01463256-S3</t>
+          <t>B01452360-I1</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>INTERIOR ALTERATION WITHIN EXISTING TENANT SPACE STE 708 ON 7TH FLOOR IN EXISTING BUILDING: MODIFY EXISTING / ADD NEW SPRINKLER HEADS PER NEW LAYOUT NO CHANGE TO OCCUPANCY, GROUP AND USE.</t>
+          <t>INSTALLATION OF NEW SIDEWALK SHED AT 207 KINGSBOROUGH 2 WALK BROOKLYN NY 11233 AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>XIU</t>
+          <t>WALIUR</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>CHEN</t>
+          <t>RAHMAN</t>
         </is>
       </c>
     </row>
@@ -2163,7 +2175,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>82-10 ROOSEVELT AVENUE, Queens</t>
+          <t>36-45 MAIN STREET, Queens</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2173,40 +2185,40 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>J &amp; G CONSTRUCTION SRVCS</t>
+          <t>MEHRAN PROPERTY MGT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Pending Plan Examiner Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>2900</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Q01462609-I1</t>
+          <t>Q01453401-I1</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>INSTALLATION OF TEMPORARY HEAVY DUTY SIDEWALK SHED AS PER PLANS. NO CHANGE IN USE, EGRESS OR OCCUPANCY. SIDEWALK SHED SHALL COMPLY WITH CHAPTER #33 OF 2022 THE NYC BUILDING CODE. LIVE LOAD 300PSF.</t>
+          <t>INSTALLATION OF AN ILLUMINATED BUSINESS ACCESSORY SIGN . NO CHANGE IN USE, EGRESS OR OCCUPANCY.</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Charles</t>
+          <t>JIN HWAN</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Davidson</t>
+          <t>CHO</t>
         </is>
       </c>
     </row>
@@ -2221,50 +2233,50 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>372 LIVINGSTON STREET, Brooklyn</t>
+          <t>61-41 SAUNDERS STREET, Queens</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Brooklyn</t>
+          <t>Queens</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Doria Scaffolding LLC</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Pending Plan Examiner Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3300</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>B01347167-P2</t>
+          <t>Q01466195-S1</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>INSTALLATION OF TEMPORARY SUSPENDED SCAFFOLDS PER PLAN SUBMITTED. WORK SHALL COMPLY WITH 2022 BUILDING CODE CHAPTER 33. NO CHANGE IN USE, EGRESS AND/OR OCCUPANCY WITH THIS APPLICATION.</t>
+          <t>RESTROOM RENOVATION</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>ZELJKO</t>
+          <t>KYEONGIL</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>STEVANOVIC</t>
+          <t>JANG</t>
         </is>
       </c>
     </row>
@@ -2279,17 +2291,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>86-17 NORTHERN BOULEVARD, Queens</t>
+          <t>218 LENOX AVENUE, Manhattan</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Queens</t>
+          <t>Manhattan</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>MK ARCHITECTURE</t>
+          <t>AFSHARI TORK PE PC</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2298,31 +2310,31 @@
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>12500</t>
+          <t>32000</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Q01464179-I1</t>
+          <t>M00831074-P1</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>The scope of work consists of Interior renovation of an existing commercial space to establish new grocery store including new ceiling, wall and floor finishes, new plumbing sinks and new storefront.</t>
+          <t>INTERIOR RENOVATION AT  BASEMENT FLOOR ONLY TO CREATE AN EATING AND DRINKING ESTABLISHMENT.  INSTALLATION OF NEW MECHANICAL SYSTEM, AND PLUMBING WORK ARE FILED UNDER SEPARATE APPLICATIONS.</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Mourad</t>
+          <t>SHAHRIAR</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Kicha</t>
+          <t>AFSHARI TORK</t>
         </is>
       </c>
     </row>
@@ -2337,17 +2349,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>82-57 241 STREET, Queens</t>
+          <t>403 WEST STREET, Manhattan</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Queens</t>
+          <t>Manhattan</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>STITCHT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2356,31 +2368,31 @@
         </is>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>14828</t>
+          <t>3750</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Q01312557-P1</t>
+          <t>M01443133-P1</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Installation of solar system on the roof as per plan. No change in use, egress or occupancy</t>
+          <t>Plumbing work for new bathroom on fourth floor.</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Ayracon</t>
+          <t>JOSEPH</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Almaraz</t>
+          <t>LOMBARDI</t>
         </is>
       </c>
     </row>
@@ -2395,7 +2407,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>1211 FLATBUSH AVENUE, Brooklyn</t>
+          <t>538 54 STREET, Brooklyn</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2414,31 +2426,31 @@
         </is>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>40000</t>
+          <t>108000</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>B01465175-I1</t>
+          <t>B01351177-P2</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Interior fit-out of tenant space of existing commercial space on the first floor. Installation of new floors. No change to use, egress or occupancy.</t>
+          <t>INSTALL NEW PLUMBING FIXTURES AT CELLAR 1ST 2ND AND 3RD FLOOR. GENERAL CONSTRUCTION WORK WAS FILED UNDER DOBNOW JOB#B01351177-I1.</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Hee Jun</t>
+          <t>JIE</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Lee</t>
+          <t>ZHU</t>
         </is>
       </c>
     </row>
@@ -2453,17 +2465,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>8709 3 AVENUE, Brooklyn</t>
+          <t>61-41 SAUNDERS STREET, Queens</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Brooklyn</t>
+          <t>Queens</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>NEC REALTY CORP</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2472,46 +2484,46 @@
         </is>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>75000</t>
+          <t>13200</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>B01461704-I1</t>
+          <t>Q01466195-I1</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Interior renovation of two existing dwelling units in a mixed use building. No change in use, egress or occupancy.</t>
+          <t>INTERIOR RENOVATION</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Ashton</t>
+          <t>KYEONGIL</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Quintin</t>
+          <t>JANG</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Alteration CO</t>
+          <t>Alteration</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>174 BEACH  120 STREET, Queens</t>
+          <t>12-27 148 STREET, Queens</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2521,65 +2533,65 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>300 AVE Y LLC</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Pending Plan Examiner Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>36450</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Q00706470-S1</t>
+          <t>Q01462113-I1</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>FILING FOR CONSTRUCTION FENCE AS PER PLANS</t>
+          <t>Installation of Solar panels on existing roof structure, No change in use, egress or occupancy.</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>JEFFREY</t>
+          <t>Chun</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>BELL</t>
+          <t>Feng</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ALT-CO - New Building with Existing Elements to Remain</t>
+          <t>Alteration</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>100 ATLANTIC AVENUE, Staten Island</t>
+          <t>241 KINGSBOROUGH    2 WALK, Brooklyn</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Staten Island</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>NYCHA</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2588,7 +2600,7 @@
         </is>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -2597,149 +2609,153 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>S01291782-S3</t>
+          <t>B01450005-I1</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>SUBSEQUENT FILING FOR MECHANICAL WORK TYPE FOR INSTALLATION OF DUCTLESS SPLIT-SYSTEM HEAT PUMPS FOR HEATING AND AIR CONDITIONING.</t>
+          <t>INSTALLATION OF NEW SIDEWALK SHED AT 241 KINGSBOROUGH 2 WALK BROOKLYN NY 11233 AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>YUNHO</t>
+          <t>WALIUR</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>LEE</t>
+          <t>RAHMAN</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Full Demolition</t>
+          <t>Alteration</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>40-38 189 STREET, Queens</t>
+          <t>6585 BROADWAY, Bronx</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Queens</t>
+          <t>Bronx</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>4038 EASTERN REALTY LLC</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Pending Plan Examiner Assignment</t>
+          <t>Pending CPE/ACPE Assignment</t>
         </is>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>45000</t>
+          <t>15000</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Q01442655-I1</t>
+          <t>X01435396-I1</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>FULLY DEMOLITION OF EXISTING 2 1/2 STORY HOUSE</t>
+          <t>Replacement of hot water heating boiler. No change in use, egress, or occupancy.</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>XIAOHONG</t>
+          <t>Yahaira</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>ZHAO</t>
+          <t>Volquez Colombo</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Alteration CO</t>
+          <t>Alteration</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>1248 HAVEMEYER AVENUE, Bronx</t>
+          <t>111 BROADWAY, Manhattan</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Bronx</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr"/>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>CAPITAL PROPERTIES</t>
+        </is>
+      </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Pending CPE/ACPE Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>200000</t>
+          <t>101200</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>X01455851-I1</t>
+          <t>M01386832-P1</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>FILING FOR INTERIOR RENOVATION WORK TO CONVERT FROM ONE FAMILY TO TWO FAMILIES.</t>
+          <t>MECHANICAL MODIFICATIONS TAKING PLACE ON 20TH FLOOR AS PER PLANS FILED HEREWITH. NO CHANGE IN USE, EGRESS, OR OCCUPANCY.</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Akeeb</t>
+          <t>Steven</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Shekoni</t>
+          <t>Snyder</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alteration CO</t>
+          <t>Alteration</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>105 BOWERY, Manhattan</t>
+          <t>301 EAST   38 STREET, Manhattan</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2749,98 +2765,906 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Bowery 87 LLC</t>
+          <t>CHESTNUT HOLDINGS</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Pending CPE/ACPE Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>150000</t>
+          <t>50000</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>M01313825-I1</t>
+          <t>M01463437-I1</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>CONVERT EXISTING INTERIM MULTIPLE DWELLING IMD)  TO OBTAIN AN AMENDED CERTIFICATE OF OCCUPANCY PER NYC LOFT BOARD REQUIREMENTS IN ACCORDANCE WITH ARTICLE 7B - NYS MULTIPLE DWELLING LAW- NO CHANGE TO EXISTING COMMERCIAL USE</t>
+          <t>FILING FOR FACADE REPIAR; REPAIR STEP CRACKS BRICK POINTING AND GRINDING AS PER PLANS. NO CHANGE IN USE, EGRESS OR OCCUPANCY.</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>MICHAEL</t>
+          <t>AKM</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>CETERA</t>
+          <t>RAHMAN</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>471 GLENMORE AVENUE, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>T&amp;J CONTRACTING INC</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Pending CPE/ACPE Assignment</t>
+        </is>
+      </c>
+      <c r="G42" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>54400</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>B01462378-I1</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>DUE TO NEW OWNER REPAIR THE EXISTING ROOF AS PER PLAN. NO CHANGE IN USE, EGRESS, OR OCCUPANCY.</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>SURESH</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>WARREN</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>133 WEST  128 STREET, Manhattan</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>AIO BUILDING CONSULTING INC</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G43" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>50000</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>M01463410-I1</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>FILING TO REPAIR AND REPLACE STUCCO AT FRONT FACADE. NO CHANGE IN USE, EGRESS OR OCCUPANCY</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>AKM</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>RAHMAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>30</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Alteration CO</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1842 HYLAN BOULEVARD, Staten Island</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Staten Island</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1838 hylan LLC</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Pending CPE/ACPE Assignment</t>
+        </is>
+      </c>
+      <c r="G44" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>500000</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>S01463126-I1</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>PROJECT TO ADD A SECOND FLOOR RESIDENTIAL SECOND FLOOR</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Mohammad</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Baalbaki</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
         <v>0</v>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>Alteration CO</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>90-01 215 STREET, Queens</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2045 EAST   14 STREET, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Pending Plan Examiner Assignment</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>15000</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>B01401287-S2</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>STRUCTURAL DESIGN IN CONJUNCTION WITH GC APPLICATION B01401287-I1</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>DAMIR</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>RAHMAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>0</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Alteration CO</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>170-07 HILLSIDE AVENUE, Queens</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
         <is>
           <t>Queens</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>Not Applicable</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>Pending Plan Examiner Assignment</t>
         </is>
       </c>
-      <c r="G42" s="1" t="n">
-        <v>46291</v>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>199150</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>Q01159189-P1</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>Extension of existing 1-family dwelling as per submitted drawing. In conjunction with BIS job#401010838. Filing to obtain a new certificate of occupancy.</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>GLEN</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>LANGER</t>
+      <c r="G46" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>20000</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Q01449931-S1</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>(PLUMBING WORK) APPLICATION FILING MINOR RENOVATION FOR EXISTING PROFESSIONAL OFFICE AND 1 FAMILY BUILDING IN CONNECTION GC JOB# Q01449931-I1. NO CHANGE TO USE, EGRESS, OCCUPANCY.</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Mohammad</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Alauddin</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>0</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Alteration CO</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>95 MADISON AVENUE, Manhattan</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>MADISON 29 HOLDING LLC</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Pending Plan Examiner Assignment</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>325000</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>M01053870-B1</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>SUBSEQUENT FILING FOR MECHANICAL WORK IN CONJUNCTION WITH ALT-CO APPLICATION # M01053870.</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>EDWIN</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>DEGUZMAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>0</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Alteration CO</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>6918 FORT HAMILTON PARKWAY, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>OM SAI REALTY LLC</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>4000</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>B01311638-S1</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>New construction wood fence along the facade on the sidewalk</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Michael</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Megalla</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>0</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Alteration CO</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>105 SOUTH    4 STREET, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Pending Plan Examiner Assignment</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>15000</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>B01311619-S5</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Support of Excavation during underpinning of adjacent building.  See plans submitted herewith and related PAA filed on DOBNOW job #B01311619-I1 filed in conjunction to document this work further per code and DOBNOW requirements.</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Michael</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Sbeglia</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>0</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Alteration CO</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2331 HERMANY AVENUE, Bronx</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Bronx</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>R and V ASSETS CORP</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Pending CPE/ACPE Assignment</t>
+        </is>
+      </c>
+      <c r="G50" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>83000</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>X01456477-I1</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Conversion of single family house to 2-family house</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Jingjun</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Zhou</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>0</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Alteration CO</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2331 GAR HERMANY AVENUE, Bronx</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Bronx</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>R and V ASSETS CORP</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Pending CPE/ACPE Assignment</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>47700</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>X01456479-I1</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>VERTICAL ENLARGEMENT OF EXISTING ONE-STORY DETACHED ACCESSORY GARAGE. NEW SECOND STORY CONTAINING ONE ANCILLARY DWELLING UNIT (477 SF) PER BC APPENDIX U. FIRST FLOOR REMAINS PRIVATE GARAGE, TWO SPACES. NEW CERTIFICATE OF OCCUPANCY. RELATED: X01456477-I1.</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Jingjun</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Zhou</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>0</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ALT-CO - New Building with Existing Elements to Remain</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>898 MADISON STREET, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ATOMIC CONTRACTING INC.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G52" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>B01216883-P7</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Install fire sprinkler system subsequent to GC (-I1) job.  The system is hydraulically calculated.</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Gregory</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Mortman</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>0</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>No Work</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>303 BOND STREET, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Pending Plan Examiner Assignment</t>
+        </is>
+      </c>
+      <c r="G53" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>B01451309-I1</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Public Programs: Lectures, Conferences, Exhibitions, Talks, Community Board Meetings</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>HAYLEY</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>EBER</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>0</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Full Demolition</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>28-17 215 PLACE, Queens</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Pending Plan Examiner Assignment</t>
+        </is>
+      </c>
+      <c r="G54" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>45000</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Q01393814-I1</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>FULLY DEMOLITION OF EXISTING 1 1/2 STORY HOUSE</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>XIAOHONG</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>ZHAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>0</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Alteration CO</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2778 MARION AVENUE, Bronx</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Bronx</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>VIDA CONSTRUCTION ENTER.</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Pending CPE/ACPE Assignment</t>
+        </is>
+      </c>
+      <c r="G55" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>188000</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>X01464167-I1</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Convert one family house to a two family house.</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Amauris</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Ramirez</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>0</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Alteration CO</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>280 HANCOCK STREET, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Pending CPE/ACPE Assignment</t>
+        </is>
+      </c>
+      <c r="G56" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>2778</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>B01242126-I1</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Change of Use for work performed in conjunction with Job #B01387834-S2.</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>MICHAEL</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>COGEN</t>
         </is>
       </c>
     </row>

</xml_diff>